<commit_message>
modified:   use it amazon.xlsx
</commit_message>
<xml_diff>
--- a/use it amazon.xlsx
+++ b/use it amazon.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7310"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7310" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="all lsiting" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="219">
   <si>
     <t>Shipment ID</t>
   </si>
@@ -620,9 +620,6 @@
     <t>Dashbord</t>
   </si>
   <si>
-    <t>M Men Style Lord Shiv B...klace For Men And women,New</t>
-  </si>
-  <si>
     <t>FBA15LSY5PTS</t>
   </si>
   <si>
@@ -675,6 +672,15 @@
   </si>
   <si>
     <t>X001VQL7BL</t>
+  </si>
+  <si>
+    <t>M Men Style</t>
+  </si>
+  <si>
+    <t>Tunglaze</t>
+  </si>
+  <si>
+    <t>Sullery</t>
   </si>
 </sst>
 </file>
@@ -1508,7 +1514,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -1623,7 +1629,7 @@
         <v>132</v>
       </c>
       <c r="D10" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E10" t="s">
         <v>17</v>
@@ -1655,7 +1661,7 @@
         <v>135</v>
       </c>
       <c r="D11" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E11" t="s">
         <v>17</v>
@@ -1687,7 +1693,7 @@
         <v>138</v>
       </c>
       <c r="D12" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E12" t="s">
         <v>17</v>
@@ -1719,7 +1725,7 @@
         <v>141</v>
       </c>
       <c r="D13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E13" t="s">
         <v>17</v>
@@ -1783,7 +1789,7 @@
         <v>144</v>
       </c>
       <c r="D15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E15" t="s">
         <v>17</v>
@@ -1815,7 +1821,7 @@
         <v>147</v>
       </c>
       <c r="D16" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E16" t="s">
         <v>17</v>
@@ -1847,7 +1853,7 @@
         <v>150</v>
       </c>
       <c r="D17" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E17" t="s">
         <v>17</v>
@@ -1879,7 +1885,7 @@
         <v>153</v>
       </c>
       <c r="D18" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E18" t="s">
         <v>17</v>
@@ -1911,7 +1917,7 @@
         <v>156</v>
       </c>
       <c r="D19" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E19" t="s">
         <v>17</v>
@@ -1943,7 +1949,7 @@
         <v>159</v>
       </c>
       <c r="D20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E20" t="s">
         <v>17</v>
@@ -1975,7 +1981,7 @@
         <v>162</v>
       </c>
       <c r="D21" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E21" t="s">
         <v>17</v>
@@ -2071,7 +2077,7 @@
         <v>165</v>
       </c>
       <c r="D24" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E24" t="s">
         <v>17</v>
@@ -2103,7 +2109,7 @@
         <v>168</v>
       </c>
       <c r="D25" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E25" t="s">
         <v>17</v>
@@ -2135,7 +2141,7 @@
         <v>171</v>
       </c>
       <c r="D26" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E26" t="s">
         <v>17</v>
@@ -2263,7 +2269,7 @@
         <v>174</v>
       </c>
       <c r="D30" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E30" t="s">
         <v>17</v>
@@ -2359,7 +2365,7 @@
         <v>177</v>
       </c>
       <c r="D33" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E33" t="s">
         <v>17</v>
@@ -2391,7 +2397,7 @@
         <v>180</v>
       </c>
       <c r="D34" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E34" t="s">
         <v>17</v>
@@ -2419,14 +2425,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.26953125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>181</v>
       </c>
@@ -2455,105 +2461,78 @@
       <c r="K1" t="s">
         <v>188</v>
       </c>
-      <c r="L1" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>191</v>
       </c>
+      <c r="B2" s="2" t="s">
+        <v>216</v>
+      </c>
       <c r="G2" t="s">
         <v>191</v>
       </c>
-      <c r="L2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>190</v>
       </c>
+      <c r="B3" s="2" t="s">
+        <v>217</v>
+      </c>
       <c r="G3" t="s">
         <v>190</v>
       </c>
-      <c r="L3" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>192</v>
       </c>
+      <c r="B4" s="2" t="s">
+        <v>218</v>
+      </c>
       <c r="G4" t="s">
         <v>192</v>
       </c>
-      <c r="L4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>193</v>
       </c>
       <c r="G5" t="s">
         <v>193</v>
       </c>
-      <c r="L5" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>194</v>
       </c>
       <c r="G6" t="s">
         <v>194</v>
       </c>
-      <c r="L6" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>195</v>
       </c>
       <c r="G7" t="s">
         <v>195</v>
       </c>
-      <c r="L7" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>196</v>
       </c>
       <c r="G8" t="s">
         <v>196</v>
       </c>
-      <c r="L8" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>197</v>
       </c>
       <c r="G9" t="s">
         <v>197</v>
-      </c>
-      <c r="L9" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="L14" t="s">
-        <v>198</v>
-      </c>
-      <c r="M14">
-        <f>LEN(L14)</f>
-        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>